<commit_message>
Update IFC parser script to match summary table format
Key features implemented:
- Modified scripts/ifc_parser.py to align materials_summary.xlsx output with summary.xlsx from extract.py
- Updated .gitignore to exclude generated Excel and JSON files in uploads directory
- Enhanced element classification logic in ifc_parser.py for more accurate categorization
- Improved material property extraction and formatting in ifc_parser.py to include detailed characteristics like concrete grade, frost resistance, and water permeability
- Adjusted summary table creation in ifc_parser.py to correctly group and display material information with proper Russian type names
- Updated JSON output in uploads/.../materials_summary.json to reflect the enhanced material details and increased number of aggregated items (from 11 to 14)

The script now produces a materials summary table with detailed material properties matching the expected format from the extract.py script.
</commit_message>
<xml_diff>
--- a/uploads/5aafc637-f347-416d-8ce7-d3c46d72772f/materials_summary.xlsx
+++ b/uploads/5aafc637-f347-416d-8ce7-d3c46d72772f/materials_summary.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Материалы" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Материалы" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,10 +433,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -496,7 +496,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Лестничные_площадки</t>
+          <t>Лестничные_марши</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -521,49 +521,49 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Пандусы</t>
+          <t>Лестничные_площадки</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>IfcRamp</t>
+          <t>IfcSlab</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Бетон В30</t>
+          <t>Бетон В25 F100 W4</t>
         </is>
       </c>
       <c r="D4" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>40</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>22.548</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Перекрытия</t>
+          <t>Пандусы</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>IfcSlab</t>
+          <t>IfcRamp</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Бетон В10</t>
+          <t>Бетон В30 F150</t>
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="E5" s="2" t="n">
-        <v>252.964</v>
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -579,14 +579,14 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Бетон В10 W6</t>
+          <t>Бетон В25 F100 W4</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>13.597</v>
+        <v>4.17</v>
       </c>
     </row>
     <row r="7">
@@ -602,14 +602,14 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Бетон В25 F100 W4</t>
+          <t>Бетон В25 F100 W6</t>
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>26.717</v>
+        <v>2242.488</v>
       </c>
     </row>
     <row r="8">
@@ -625,14 +625,14 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Бетон В25 F100 W6</t>
+          <t>Бетон В30 F150 W6</t>
         </is>
       </c>
       <c r="D8" s="2" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>2242.488</v>
+        <v>982.649</v>
       </c>
     </row>
     <row r="9">
@@ -648,20 +648,20 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Бетон В30 F150 W6</t>
+          <t>Бетон В35 F150 W6</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>2139.742</v>
+        <v>453.753</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Перекрытия</t>
+          <t>Подготовка_фундамента</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -671,37 +671,37 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Бетон В35 F150 W6</t>
+          <t>Бетон В10</t>
         </is>
       </c>
       <c r="D10" s="2" t="n">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1147.493</v>
+        <v>252.964</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Стены</t>
+          <t>Подготовка_фундамента</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>IfcWall</t>
+          <t>IfcSlab</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Бетон В30 F150 W6</t>
+          <t>Бетон В10 W6</t>
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>984</v>
+        <v>1</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1731.541</v>
+        <v>13.597</v>
       </c>
     </row>
     <row r="12">
@@ -717,14 +717,83 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
+          <t>Бетон В30 F150 W6</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>984</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>1731.541</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Стены</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>IfcWall</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
           <t>Бетон В35 F150 W6</t>
         </is>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D13" s="2" t="n">
         <v>163</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E13" s="2" t="n">
         <v>607.577</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Фундаментные_плиты</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>IfcSlab</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В30 F150 W6</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1157.093</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Фундаментные_плиты</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>IfcSlab</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Бетон В35 F150 W6</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>693.739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>